<commit_message>
Improve HRIS demo and project documentation
</commit_message>
<xml_diff>
--- a/config/mapping_config.xlsx
+++ b/config/mapping_config.xlsx
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1407,6 +1407,66 @@
       <c r="F25" t="inlineStr">
         <is>
           <t>有效邮箱直接映射</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">离职 </t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>RESIGN</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Demo 模式使用预先确认的值映射</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>休假</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>L-ACTIVE</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="E27" t="b">
+        <v>0</v>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Demo 模式使用预先确认的值映射</t>
         </is>
       </c>
     </row>

</xml_diff>